<commit_message>
Dashboard --base-url + файлы лотов
</commit_message>
<xml_diff>
--- a/vse-loti/340581586/spec-340581586.xlsx
+++ b/vse-loti/340581586/spec-340581586.xlsx
@@ -84,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -97,6 +97,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -465,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -558,7 +561,7 @@
         <v>1824726.91</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>2189672.29</v>
+        <v>2226166.83</v>
       </c>
     </row>
     <row r="3">
@@ -593,7 +596,7 @@
         <v>269558.86</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>323470.63</v>
+        <v>328861.81</v>
       </c>
     </row>
     <row r="4">
@@ -628,7 +631,7 @@
         <v>506051.15</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>607261.38</v>
+        <v>617382.41</v>
       </c>
     </row>
     <row r="5">
@@ -663,7 +666,7 @@
         <v>230174.52</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>276209.42</v>
+        <v>280812.91</v>
       </c>
     </row>
     <row r="6">
@@ -698,7 +701,7 @@
         <v>759530.9399999999</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>911437.13</v>
+        <v>926627.75</v>
       </c>
     </row>
     <row r="7">
@@ -733,7 +736,7 @@
         <v>98269.16</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>117922.99</v>
+        <v>119888.38</v>
       </c>
     </row>
     <row r="8">
@@ -768,7 +771,7 @@
         <v>573338.21</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>688005.85</v>
+        <v>699472.61</v>
       </c>
     </row>
     <row r="9">
@@ -803,7 +806,7 @@
         <v>573338.21</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>688005.85</v>
+        <v>699472.61</v>
       </c>
     </row>
     <row r="10">
@@ -838,7 +841,7 @@
         <v>398416.83</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>478100.2</v>
+        <v>486068.53</v>
       </c>
     </row>
     <row r="11">
@@ -873,7 +876,7 @@
         <v>398416.83</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>478100.2</v>
+        <v>486068.53</v>
       </c>
     </row>
     <row r="12">
@@ -908,7 +911,7 @@
         <v>398416.83</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>478100.2</v>
+        <v>486068.53</v>
       </c>
     </row>
     <row r="13">
@@ -943,7 +946,7 @@
         <v>398416.83</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>478100.2</v>
+        <v>486068.53</v>
       </c>
     </row>
     <row r="14">
@@ -978,7 +981,7 @@
         <v>398416.83</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>478100.2</v>
+        <v>486068.53</v>
       </c>
     </row>
     <row r="15">
@@ -1013,7 +1016,7 @@
         <v>129801.73</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>155762.07</v>
+        <v>158358.11</v>
       </c>
     </row>
     <row r="16">
@@ -1048,7 +1051,7 @@
         <v>161817.29</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>194180.75</v>
+        <v>197417.09</v>
       </c>
     </row>
     <row r="17">
@@ -1083,7 +1086,7 @@
         <v>206845.12</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>248214.15</v>
+        <v>252351.05</v>
       </c>
     </row>
     <row r="18">
@@ -1118,7 +1121,7 @@
         <v>367994.37</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>441593.24</v>
+        <v>448953.13</v>
       </c>
     </row>
     <row r="19">
@@ -1153,7 +1156,7 @@
         <v>102299.52</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>122759.43</v>
+        <v>124805.42</v>
       </c>
     </row>
     <row r="20">
@@ -1188,7 +1191,7 @@
         <v>1824726.91</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>2189672.29</v>
+        <v>2226166.83</v>
       </c>
     </row>
     <row r="21">
@@ -1223,7 +1226,7 @@
         <v>412405.42</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>494886.5</v>
+        <v>503134.61</v>
       </c>
     </row>
     <row r="22">
@@ -1258,7 +1261,7 @@
         <v>185767.06</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>222920.47</v>
+        <v>226635.81</v>
       </c>
     </row>
     <row r="23">
@@ -1293,7 +1296,7 @@
         <v>769537.49</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>923444.98</v>
+        <v>938835.73</v>
       </c>
     </row>
     <row r="24">
@@ -1328,7 +1331,7 @@
         <v>366332.1</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>439598.52</v>
+        <v>446925.16</v>
       </c>
     </row>
     <row r="25">
@@ -1363,7 +1366,7 @@
         <v>398155.39</v>
       </c>
       <c r="I25" s="5" t="n">
-        <v>477786.47</v>
+        <v>485749.57</v>
       </c>
     </row>
     <row r="26">
@@ -1398,7 +1401,7 @@
         <v>398155.39</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>477786.47</v>
+        <v>485749.57</v>
       </c>
     </row>
     <row r="27">
@@ -1433,7 +1436,7 @@
         <v>398155.39</v>
       </c>
       <c r="I27" s="5" t="n">
-        <v>477786.47</v>
+        <v>485749.57</v>
       </c>
     </row>
     <row r="28">
@@ -1468,7 +1471,7 @@
         <v>398155.39</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>477786.47</v>
+        <v>485749.57</v>
       </c>
     </row>
     <row r="29">
@@ -1503,7 +1506,7 @@
         <v>849273.28</v>
       </c>
       <c r="I29" s="5" t="n">
-        <v>1019127.93</v>
+        <v>1036113.4</v>
       </c>
     </row>
     <row r="30">
@@ -1538,7 +1541,7 @@
         <v>114613.29</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>137535.95</v>
+        <v>139828.22</v>
       </c>
     </row>
     <row r="31">
@@ -1573,7 +1576,7 @@
         <v>298735.98</v>
       </c>
       <c r="I31" s="5" t="n">
-        <v>358483.18</v>
+        <v>364457.9</v>
       </c>
     </row>
     <row r="32">
@@ -1608,7 +1611,7 @@
         <v>341818.11</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>410181.73</v>
+        <v>417018.09</v>
       </c>
     </row>
     <row r="33">
@@ -1643,7 +1646,7 @@
         <v>102299.52</v>
       </c>
       <c r="I33" s="5" t="n">
-        <v>122759.43</v>
+        <v>124805.42</v>
       </c>
     </row>
     <row r="34">
@@ -1678,7 +1681,7 @@
         <v>173234.63</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>207881.55</v>
+        <v>211346.25</v>
       </c>
     </row>
     <row r="35">
@@ -1713,7 +1716,7 @@
         <v>206845.12</v>
       </c>
       <c r="I35" s="5" t="n">
-        <v>248214.15</v>
+        <v>252351.05</v>
       </c>
     </row>
     <row r="36">
@@ -1748,7 +1751,7 @@
         <v>406310.26</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>487572.32</v>
+        <v>495698.52</v>
       </c>
     </row>
     <row r="37">
@@ -1783,7 +1786,7 @@
         <v>254918.9</v>
       </c>
       <c r="I37" s="5" t="n">
-        <v>305902.68</v>
+        <v>311001.06</v>
       </c>
     </row>
     <row r="38">
@@ -1818,7 +1821,7 @@
         <v>151413.39</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>181696.06</v>
+        <v>184724.33</v>
       </c>
     </row>
     <row r="39">
@@ -1853,7 +1856,7 @@
         <v>183150.36</v>
       </c>
       <c r="I39" s="5" t="n">
-        <v>219780.43</v>
+        <v>223443.44</v>
       </c>
     </row>
     <row r="40">
@@ -1888,7 +1891,7 @@
         <v>211307.22</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>253568.66</v>
+        <v>257794.81</v>
       </c>
     </row>
     <row r="41">
@@ -1923,7 +1926,7 @@
         <v>254230.2</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>305076.24</v>
+        <v>310160.84</v>
       </c>
     </row>
     <row r="42">
@@ -1958,7 +1961,7 @@
         <v>102299.52</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>122759.43</v>
+        <v>124805.42</v>
       </c>
     </row>
     <row r="43">
@@ -1993,7 +1996,7 @@
         <v>1399301.6</v>
       </c>
       <c r="I43" s="5" t="n">
-        <v>1679161.92</v>
+        <v>1707147.95</v>
       </c>
     </row>
     <row r="44">
@@ -2019,18 +2022,35 @@
         <v>2495555.9673</v>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>НМЦК с НДС 22% (справочно):</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="n">
+        <v>3044578.28</v>
+      </c>
+    </row>
     <row r="47">
       <c r="A47" s="10" t="inlineStr">
         <is>
+          <t>Ставка НДС в документах не указана, расчёт справочный по 22 %; суммы источника указаны без НДС: "Цена за единицу продукции (без НДС) р." — Задание на закупку Труба стальная.txt. «без НДС» — сумма из документа, «с НДС» = сумма × 1,22.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="11" t="inlineStr">
+        <is>
           <t>Источник: Задание на закупку Труба стальная.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="48"/>
-    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A47:B49"/>
+    <mergeCell ref="A49:B51"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Dashboard 2026-09-24 + файлы лотов
</commit_message>
<xml_diff>
--- a/vse-loti/340581586/spec-340581586.xlsx
+++ b/vse-loti/340581586/spec-340581586.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:J51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -480,6 +480,7 @@
     <col width="20.28515625" customWidth="1" min="7" max="7"/>
     <col width="18.85546875" customWidth="1" min="8" max="8"/>
     <col width="16.42578125" customWidth="1" min="9" max="9"/>
+    <col width="18.85546875" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -515,17 +516,22 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Цена за т (без НДС)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Стоимость (без НДС)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Цена за т (без НДС)</t>
-        </is>
-      </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Цена за т (с НДС)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Стоимость (с НДС)</t>
         </is>
       </c>
     </row>
@@ -555,13 +561,16 @@
         <v>0.017</v>
       </c>
       <c r="G2" s="5" t="n">
+        <v>1824726.91</v>
+      </c>
+      <c r="H2" s="5" t="n">
         <v>30870</v>
-      </c>
-      <c r="H2" s="5" t="n">
-        <v>1824726.91</v>
       </c>
       <c r="I2" s="5" t="n">
         <v>2226166.83</v>
+      </c>
+      <c r="J2" s="5" t="n">
+        <v>37661.4</v>
       </c>
     </row>
     <row r="3">
@@ -590,13 +599,16 @@
         <v>0.368</v>
       </c>
       <c r="G3" s="5" t="n">
+        <v>269558.86</v>
+      </c>
+      <c r="H3" s="5" t="n">
         <v>99077.75999999999</v>
-      </c>
-      <c r="H3" s="5" t="n">
-        <v>269558.86</v>
       </c>
       <c r="I3" s="5" t="n">
         <v>328861.81</v>
+      </c>
+      <c r="J3" s="5" t="n">
+        <v>120874.87</v>
       </c>
     </row>
     <row r="4">
@@ -625,13 +637,16 @@
         <v>0.012</v>
       </c>
       <c r="G4" s="5" t="n">
+        <v>506051.15</v>
+      </c>
+      <c r="H4" s="5" t="n">
         <v>5840.64</v>
-      </c>
-      <c r="H4" s="5" t="n">
-        <v>506051.15</v>
       </c>
       <c r="I4" s="5" t="n">
         <v>617382.41</v>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>7125.58</v>
       </c>
     </row>
     <row r="5">
@@ -660,13 +675,16 @@
         <v>0.078</v>
       </c>
       <c r="G5" s="5" t="n">
+        <v>230174.52</v>
+      </c>
+      <c r="H5" s="5" t="n">
         <v>17937.5</v>
-      </c>
-      <c r="H5" s="5" t="n">
-        <v>230174.52</v>
       </c>
       <c r="I5" s="5" t="n">
         <v>280812.91</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>21883.75</v>
       </c>
     </row>
     <row r="6">
@@ -695,13 +713,16 @@
         <v>0.023</v>
       </c>
       <c r="G6" s="5" t="n">
+        <v>759530.9399999999</v>
+      </c>
+      <c r="H6" s="5" t="n">
         <v>17643.6</v>
-      </c>
-      <c r="H6" s="5" t="n">
-        <v>759530.9399999999</v>
       </c>
       <c r="I6" s="5" t="n">
         <v>926627.75</v>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>21525.19</v>
       </c>
     </row>
     <row r="7">
@@ -730,13 +751,16 @@
         <v>0.384</v>
       </c>
       <c r="G7" s="5" t="n">
+        <v>98269.16</v>
+      </c>
+      <c r="H7" s="5" t="n">
         <v>37689.84</v>
-      </c>
-      <c r="H7" s="5" t="n">
-        <v>98269.16</v>
       </c>
       <c r="I7" s="5" t="n">
         <v>119888.38</v>
+      </c>
+      <c r="J7" s="5" t="n">
+        <v>45981.6</v>
       </c>
     </row>
     <row r="8">
@@ -765,13 +789,16 @@
         <v>0.164</v>
       </c>
       <c r="G8" s="5" t="n">
+        <v>573338.21</v>
+      </c>
+      <c r="H8" s="5" t="n">
         <v>94119.2</v>
-      </c>
-      <c r="H8" s="5" t="n">
-        <v>573338.21</v>
       </c>
       <c r="I8" s="5" t="n">
         <v>699472.61</v>
+      </c>
+      <c r="J8" s="5" t="n">
+        <v>114825.42</v>
       </c>
     </row>
     <row r="9">
@@ -800,13 +827,16 @@
         <v>0.082</v>
       </c>
       <c r="G9" s="5" t="n">
+        <v>573338.21</v>
+      </c>
+      <c r="H9" s="5" t="n">
         <v>47059.6</v>
-      </c>
-      <c r="H9" s="5" t="n">
-        <v>573338.21</v>
       </c>
       <c r="I9" s="5" t="n">
         <v>699472.61</v>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>57412.71</v>
       </c>
     </row>
     <row r="10">
@@ -835,13 +865,16 @@
         <v>0.885</v>
       </c>
       <c r="G10" s="5" t="n">
+        <v>398416.83</v>
+      </c>
+      <c r="H10" s="5" t="n">
         <v>352696.64</v>
-      </c>
-      <c r="H10" s="5" t="n">
-        <v>398416.83</v>
       </c>
       <c r="I10" s="5" t="n">
         <v>486068.53</v>
+      </c>
+      <c r="J10" s="5" t="n">
+        <v>430289.9</v>
       </c>
     </row>
     <row r="11">
@@ -870,13 +903,16 @@
         <v>0.032</v>
       </c>
       <c r="G11" s="5" t="n">
+        <v>398416.83</v>
+      </c>
+      <c r="H11" s="5" t="n">
         <v>12733.88</v>
-      </c>
-      <c r="H11" s="5" t="n">
-        <v>398416.83</v>
       </c>
       <c r="I11" s="5" t="n">
         <v>486068.53</v>
+      </c>
+      <c r="J11" s="5" t="n">
+        <v>15535.33</v>
       </c>
     </row>
     <row r="12">
@@ -905,13 +941,16 @@
         <v>0.07199999999999999</v>
       </c>
       <c r="G12" s="5" t="n">
+        <v>398416.83</v>
+      </c>
+      <c r="H12" s="5" t="n">
         <v>28651.23</v>
-      </c>
-      <c r="H12" s="5" t="n">
-        <v>398416.83</v>
       </c>
       <c r="I12" s="5" t="n">
         <v>486068.53</v>
+      </c>
+      <c r="J12" s="5" t="n">
+        <v>34954.5</v>
       </c>
     </row>
     <row r="13">
@@ -940,13 +979,16 @@
         <v>0.07199999999999999</v>
       </c>
       <c r="G13" s="5" t="n">
+        <v>398416.83</v>
+      </c>
+      <c r="H13" s="5" t="n">
         <v>28651.23</v>
-      </c>
-      <c r="H13" s="5" t="n">
-        <v>398416.83</v>
       </c>
       <c r="I13" s="5" t="n">
         <v>486068.53</v>
+      </c>
+      <c r="J13" s="5" t="n">
+        <v>34954.5</v>
       </c>
     </row>
     <row r="14">
@@ -975,13 +1017,16 @@
         <v>0.639</v>
       </c>
       <c r="G14" s="5" t="n">
+        <v>398416.83</v>
+      </c>
+      <c r="H14" s="5" t="n">
         <v>254677.6</v>
-      </c>
-      <c r="H14" s="5" t="n">
-        <v>398416.83</v>
       </c>
       <c r="I14" s="5" t="n">
         <v>486068.53</v>
+      </c>
+      <c r="J14" s="5" t="n">
+        <v>310706.67</v>
       </c>
     </row>
     <row r="15">
@@ -1010,13 +1055,16 @@
         <v>0.5</v>
       </c>
       <c r="G15" s="5" t="n">
+        <v>129801.73</v>
+      </c>
+      <c r="H15" s="5" t="n">
         <v>64942.4</v>
-      </c>
-      <c r="H15" s="5" t="n">
-        <v>129801.73</v>
       </c>
       <c r="I15" s="5" t="n">
         <v>158358.11</v>
+      </c>
+      <c r="J15" s="5" t="n">
+        <v>79229.73</v>
       </c>
     </row>
     <row r="16">
@@ -1045,13 +1093,16 @@
         <v>0.74</v>
       </c>
       <c r="G16" s="5" t="n">
+        <v>161817.29</v>
+      </c>
+      <c r="H16" s="5" t="n">
         <v>119809.52</v>
-      </c>
-      <c r="H16" s="5" t="n">
-        <v>161817.29</v>
       </c>
       <c r="I16" s="5" t="n">
         <v>197417.09</v>
+      </c>
+      <c r="J16" s="5" t="n">
+        <v>146167.61</v>
       </c>
     </row>
     <row r="17">
@@ -1080,13 +1131,16 @@
         <v>0.126</v>
       </c>
       <c r="G17" s="5" t="n">
+        <v>206845.12</v>
+      </c>
+      <c r="H17" s="5" t="n">
         <v>25963.2</v>
-      </c>
-      <c r="H17" s="5" t="n">
-        <v>206845.12</v>
       </c>
       <c r="I17" s="5" t="n">
         <v>252351.05</v>
+      </c>
+      <c r="J17" s="5" t="n">
+        <v>31675.1</v>
       </c>
     </row>
     <row r="18">
@@ -1115,13 +1169,16 @@
         <v>0.17</v>
       </c>
       <c r="G18" s="5" t="n">
+        <v>367994.37</v>
+      </c>
+      <c r="H18" s="5" t="n">
         <v>62706.24</v>
-      </c>
-      <c r="H18" s="5" t="n">
-        <v>367994.37</v>
       </c>
       <c r="I18" s="5" t="n">
         <v>448953.13</v>
+      </c>
+      <c r="J18" s="5" t="n">
+        <v>76501.61</v>
       </c>
     </row>
     <row r="19">
@@ -1150,13 +1207,16 @@
         <v>0.268</v>
       </c>
       <c r="G19" s="5" t="n">
+        <v>102299.52</v>
+      </c>
+      <c r="H19" s="5" t="n">
         <v>27432.64</v>
-      </c>
-      <c r="H19" s="5" t="n">
-        <v>102299.52</v>
       </c>
       <c r="I19" s="5" t="n">
         <v>124805.42</v>
+      </c>
+      <c r="J19" s="5" t="n">
+        <v>33467.82</v>
       </c>
     </row>
     <row r="20">
@@ -1185,13 +1245,16 @@
         <v>0.017</v>
       </c>
       <c r="G20" s="5" t="n">
+        <v>1824726.91</v>
+      </c>
+      <c r="H20" s="5" t="n">
         <v>30870</v>
-      </c>
-      <c r="H20" s="5" t="n">
-        <v>1824726.91</v>
       </c>
       <c r="I20" s="5" t="n">
         <v>2226166.83</v>
+      </c>
+      <c r="J20" s="5" t="n">
+        <v>37661.4</v>
       </c>
     </row>
     <row r="21">
@@ -1220,13 +1283,16 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="G21" s="5" t="n">
+        <v>412405.42</v>
+      </c>
+      <c r="H21" s="5" t="n">
         <v>36451.36</v>
-      </c>
-      <c r="H21" s="5" t="n">
-        <v>412405.42</v>
       </c>
       <c r="I21" s="5" t="n">
         <v>503134.61</v>
+      </c>
+      <c r="J21" s="5" t="n">
+        <v>44470.66</v>
       </c>
     </row>
     <row r="22">
@@ -1255,13 +1321,16 @@
         <v>0.328</v>
       </c>
       <c r="G22" s="5" t="n">
+        <v>185767.06</v>
+      </c>
+      <c r="H22" s="5" t="n">
         <v>60991.04</v>
-      </c>
-      <c r="H22" s="5" t="n">
-        <v>185767.06</v>
       </c>
       <c r="I22" s="5" t="n">
         <v>226635.81</v>
+      </c>
+      <c r="J22" s="5" t="n">
+        <v>74409.07000000001</v>
       </c>
     </row>
     <row r="23">
@@ -1290,13 +1359,16 @@
         <v>0.019</v>
       </c>
       <c r="G23" s="5" t="n">
+        <v>769537.49</v>
+      </c>
+      <c r="H23" s="5" t="n">
         <v>14575.04</v>
-      </c>
-      <c r="H23" s="5" t="n">
-        <v>769537.49</v>
       </c>
       <c r="I23" s="5" t="n">
         <v>938835.73</v>
+      </c>
+      <c r="J23" s="5" t="n">
+        <v>17781.55</v>
       </c>
     </row>
     <row r="24">
@@ -1325,13 +1397,16 @@
         <v>0.1</v>
       </c>
       <c r="G24" s="5" t="n">
+        <v>366332.1</v>
+      </c>
+      <c r="H24" s="5" t="n">
         <v>36589.25</v>
-      </c>
-      <c r="H24" s="5" t="n">
-        <v>366332.1</v>
       </c>
       <c r="I24" s="5" t="n">
         <v>446925.16</v>
+      </c>
+      <c r="J24" s="5" t="n">
+        <v>44638.89</v>
       </c>
     </row>
     <row r="25">
@@ -1360,13 +1435,16 @@
         <v>0.012</v>
       </c>
       <c r="G25" s="5" t="n">
+        <v>398155.39</v>
+      </c>
+      <c r="H25" s="5" t="n">
         <v>4618.93</v>
-      </c>
-      <c r="H25" s="5" t="n">
-        <v>398155.39</v>
       </c>
       <c r="I25" s="5" t="n">
         <v>485749.57</v>
+      </c>
+      <c r="J25" s="5" t="n">
+        <v>5635.09</v>
       </c>
     </row>
     <row r="26">
@@ -1395,13 +1473,16 @@
         <v>0.012</v>
       </c>
       <c r="G26" s="5" t="n">
+        <v>398155.39</v>
+      </c>
+      <c r="H26" s="5" t="n">
         <v>4618.93</v>
-      </c>
-      <c r="H26" s="5" t="n">
-        <v>398155.39</v>
       </c>
       <c r="I26" s="5" t="n">
         <v>485749.57</v>
+      </c>
+      <c r="J26" s="5" t="n">
+        <v>5635.09</v>
       </c>
     </row>
     <row r="27">
@@ -1430,13 +1511,16 @@
         <v>0.012</v>
       </c>
       <c r="G27" s="5" t="n">
+        <v>398155.39</v>
+      </c>
+      <c r="H27" s="5" t="n">
         <v>4618.93</v>
-      </c>
-      <c r="H27" s="5" t="n">
-        <v>398155.39</v>
       </c>
       <c r="I27" s="5" t="n">
         <v>485749.57</v>
+      </c>
+      <c r="J27" s="5" t="n">
+        <v>5635.09</v>
       </c>
     </row>
     <row r="28">
@@ -1465,13 +1549,16 @@
         <v>0.012</v>
       </c>
       <c r="G28" s="5" t="n">
+        <v>398155.39</v>
+      </c>
+      <c r="H28" s="5" t="n">
         <v>4618.93</v>
-      </c>
-      <c r="H28" s="5" t="n">
-        <v>398155.39</v>
       </c>
       <c r="I28" s="5" t="n">
         <v>485749.57</v>
+      </c>
+      <c r="J28" s="5" t="n">
+        <v>5635.09</v>
       </c>
     </row>
     <row r="29">
@@ -1500,13 +1587,16 @@
         <v>0.017</v>
       </c>
       <c r="G29" s="5" t="n">
+        <v>849273.28</v>
+      </c>
+      <c r="H29" s="5" t="n">
         <v>14163.84</v>
-      </c>
-      <c r="H29" s="5" t="n">
-        <v>849273.28</v>
       </c>
       <c r="I29" s="5" t="n">
         <v>1036113.4</v>
+      </c>
+      <c r="J29" s="5" t="n">
+        <v>17279.88</v>
       </c>
     </row>
     <row r="30">
@@ -1535,13 +1625,16 @@
         <v>0.509</v>
       </c>
       <c r="G30" s="5" t="n">
+        <v>114613.29</v>
+      </c>
+      <c r="H30" s="5" t="n">
         <v>58340</v>
-      </c>
-      <c r="H30" s="5" t="n">
-        <v>114613.29</v>
       </c>
       <c r="I30" s="5" t="n">
         <v>139828.22</v>
+      </c>
+      <c r="J30" s="5" t="n">
+        <v>71174.8</v>
       </c>
     </row>
     <row r="31">
@@ -1570,13 +1663,16 @@
         <v>0.607</v>
       </c>
       <c r="G31" s="5" t="n">
+        <v>298735.98</v>
+      </c>
+      <c r="H31" s="5" t="n">
         <v>181413.52</v>
-      </c>
-      <c r="H31" s="5" t="n">
-        <v>298735.98</v>
       </c>
       <c r="I31" s="5" t="n">
         <v>364457.9</v>
+      </c>
+      <c r="J31" s="5" t="n">
+        <v>221324.49</v>
       </c>
     </row>
     <row r="32">
@@ -1605,13 +1701,16 @@
         <v>0.203</v>
       </c>
       <c r="G32" s="5" t="n">
+        <v>341818.11</v>
+      </c>
+      <c r="H32" s="5" t="n">
         <v>69457.44</v>
-      </c>
-      <c r="H32" s="5" t="n">
-        <v>341818.11</v>
       </c>
       <c r="I32" s="5" t="n">
         <v>417018.09</v>
+      </c>
+      <c r="J32" s="5" t="n">
+        <v>84738.08</v>
       </c>
     </row>
     <row r="33">
@@ -1640,13 +1739,16 @@
         <v>0.469</v>
       </c>
       <c r="G33" s="5" t="n">
+        <v>102299.52</v>
+      </c>
+      <c r="H33" s="5" t="n">
         <v>48007.12</v>
-      </c>
-      <c r="H33" s="5" t="n">
-        <v>102299.52</v>
       </c>
       <c r="I33" s="5" t="n">
         <v>124805.42</v>
+      </c>
+      <c r="J33" s="5" t="n">
+        <v>58568.69</v>
       </c>
     </row>
     <row r="34">
@@ -1675,13 +1777,16 @@
         <v>0.15</v>
       </c>
       <c r="G34" s="5" t="n">
+        <v>173234.63</v>
+      </c>
+      <c r="H34" s="5" t="n">
         <v>25974.8</v>
-      </c>
-      <c r="H34" s="5" t="n">
-        <v>173234.63</v>
       </c>
       <c r="I34" s="5" t="n">
         <v>211346.25</v>
+      </c>
+      <c r="J34" s="5" t="n">
+        <v>31689.26</v>
       </c>
     </row>
     <row r="35">
@@ -1710,13 +1815,16 @@
         <v>0.293</v>
       </c>
       <c r="G35" s="5" t="n">
+        <v>206845.12</v>
+      </c>
+      <c r="H35" s="5" t="n">
         <v>60580.8</v>
-      </c>
-      <c r="H35" s="5" t="n">
-        <v>206845.12</v>
       </c>
       <c r="I35" s="5" t="n">
         <v>252351.05</v>
+      </c>
+      <c r="J35" s="5" t="n">
+        <v>73908.58</v>
       </c>
     </row>
     <row r="36">
@@ -1745,13 +1853,16 @@
         <v>0.134</v>
       </c>
       <c r="G36" s="5" t="n">
+        <v>406310.26</v>
+      </c>
+      <c r="H36" s="5" t="n">
         <v>54478.08</v>
-      </c>
-      <c r="H36" s="5" t="n">
-        <v>406310.26</v>
       </c>
       <c r="I36" s="5" t="n">
         <v>495698.52</v>
+      </c>
+      <c r="J36" s="5" t="n">
+        <v>66463.25999999999</v>
       </c>
     </row>
     <row r="37">
@@ -1780,13 +1891,16 @@
         <v>0.305</v>
       </c>
       <c r="G37" s="5" t="n">
+        <v>254918.9</v>
+      </c>
+      <c r="H37" s="5" t="n">
         <v>77699.28</v>
-      </c>
-      <c r="H37" s="5" t="n">
-        <v>254918.9</v>
       </c>
       <c r="I37" s="5" t="n">
         <v>311001.06</v>
+      </c>
+      <c r="J37" s="5" t="n">
+        <v>94793.12</v>
       </c>
     </row>
     <row r="38">
@@ -1815,13 +1929,16 @@
         <v>0.508</v>
       </c>
       <c r="G38" s="5" t="n">
+        <v>151413.39</v>
+      </c>
+      <c r="H38" s="5" t="n">
         <v>76918</v>
-      </c>
-      <c r="H38" s="5" t="n">
-        <v>151413.39</v>
       </c>
       <c r="I38" s="5" t="n">
         <v>184724.33</v>
+      </c>
+      <c r="J38" s="5" t="n">
+        <v>93839.96000000001</v>
       </c>
     </row>
     <row r="39">
@@ -1850,13 +1967,16 @@
         <v>0.067</v>
       </c>
       <c r="G39" s="5" t="n">
+        <v>183150.36</v>
+      </c>
+      <c r="H39" s="5" t="n">
         <v>12278.4</v>
-      </c>
-      <c r="H39" s="5" t="n">
-        <v>183150.36</v>
       </c>
       <c r="I39" s="5" t="n">
         <v>223443.44</v>
+      </c>
+      <c r="J39" s="5" t="n">
+        <v>14979.65</v>
       </c>
     </row>
     <row r="40">
@@ -1885,13 +2005,16 @@
         <v>0.505</v>
       </c>
       <c r="G40" s="5" t="n">
+        <v>211307.22</v>
+      </c>
+      <c r="H40" s="5" t="n">
         <v>106734.32</v>
-      </c>
-      <c r="H40" s="5" t="n">
-        <v>211307.22</v>
       </c>
       <c r="I40" s="5" t="n">
         <v>257794.81</v>
+      </c>
+      <c r="J40" s="5" t="n">
+        <v>130215.87</v>
       </c>
     </row>
     <row r="41">
@@ -1920,13 +2043,16 @@
         <v>0.019</v>
       </c>
       <c r="G41" s="5" t="n">
+        <v>254230.2</v>
+      </c>
+      <c r="H41" s="5" t="n">
         <v>4815.12</v>
-      </c>
-      <c r="H41" s="5" t="n">
-        <v>254230.2</v>
       </c>
       <c r="I41" s="5" t="n">
         <v>310160.84</v>
+      </c>
+      <c r="J41" s="5" t="n">
+        <v>5874.45</v>
       </c>
     </row>
     <row r="42">
@@ -1955,13 +2081,16 @@
         <v>0.469</v>
       </c>
       <c r="G42" s="5" t="n">
+        <v>102299.52</v>
+      </c>
+      <c r="H42" s="5" t="n">
         <v>48007.12</v>
-      </c>
-      <c r="H42" s="5" t="n">
-        <v>102299.52</v>
       </c>
       <c r="I42" s="5" t="n">
         <v>124805.42</v>
+      </c>
+      <c r="J42" s="5" t="n">
+        <v>58568.69</v>
       </c>
     </row>
     <row r="43">
@@ -1990,14 +2119,17 @@
         <v>0.093</v>
       </c>
       <c r="G43" s="5" t="n">
+        <v>1399301.6</v>
+      </c>
+      <c r="H43" s="5" t="n">
         <v>130233</v>
-      </c>
-      <c r="H43" s="5" t="n">
-        <v>1399301.6</v>
       </c>
       <c r="I43" s="5" t="n">
         <v>1707147.95</v>
       </c>
+      <c r="J43" s="5" t="n">
+        <v>158884.26</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -2009,7 +2141,16 @@
         <v>9.58</v>
       </c>
       <c r="G44" s="9" t="n">
+        <v>260496.45</v>
+      </c>
+      <c r="H44" s="9" t="n">
         <v>2495555.97</v>
+      </c>
+      <c r="I44" s="9" t="n">
+        <v>317805.67</v>
+      </c>
+      <c r="J44" s="9" t="n">
+        <v>3044578.28</v>
       </c>
     </row>
     <row r="45">
@@ -2018,7 +2159,7 @@
           <t>НМЦК из обоснования:</t>
         </is>
       </c>
-      <c r="G45" s="9" t="n">
+      <c r="H45" s="9" t="n">
         <v>2495555.9673</v>
       </c>
     </row>
@@ -2028,7 +2169,7 @@
           <t>НМЦК с НДС 22% (справочно):</t>
         </is>
       </c>
-      <c r="F46" s="9" t="n">
+      <c r="J46" s="9" t="n">
         <v>3044578.28</v>
       </c>
     </row>

</xml_diff>